<commit_message>
updated contact in test xlsx
</commit_message>
<xml_diff>
--- a/spec/fixtures/batch_submission_manifest_errors_columns.xlsx
+++ b/spec/fixtures/batch_submission_manifest_errors_columns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/Desktop/scripts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/spec/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFCC26A-5271-D04B-B6D4-7367040305D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364DA35D-126F-1046-88D1-7666EDF6DB10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2380" yWindow="1000" windowWidth="27640" windowHeight="15740" xr2:uid="{B67D321E-7C1E-1B4C-B0D3-48C3E7F2330E}"/>
   </bookViews>

</xml_diff>

<commit_message>
remove publication_status from manifest file
</commit_message>
<xml_diff>
--- a/spec/fixtures/batch_submission_manifest_errors_columns.xlsx
+++ b/spec/fixtures/batch_submission_manifest_errors_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/spec/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2300A489-3D31-CD4C-9F73-7EB6672D400B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3896FF05-6D15-A947-AE64-F70F7D1ED464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2380" yWindow="1000" windowWidth="27640" windowHeight="15740" xr2:uid="{B67D321E-7C1E-1B4C-B0D3-48C3E7F2330E}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="246">
   <si>
     <t>Field Section</t>
   </si>
@@ -500,11 +500,6 @@
     </r>
   </si>
   <si>
-    <t>Open: Published with Open Download
-RestrictedDownload: Published with Restricted Download
-Private: Private</t>
-  </si>
-  <si>
     <t>CTImageSeries: CT/MRI image series (multiple files of type *.tiff, *.png, *.dcm, *.zip, etc.)
 Image: Image (*.tiff, *.png, *.dcm, etc.)
 Mesh: Mesh or point cloud (*.stl, *.ply, .etc, with optional associated texture or color file)
@@ -591,9 +586,6 @@
   </si>
   <si>
     <t>media.preview_file</t>
-  </si>
-  <si>
-    <t>media.publication_status</t>
   </si>
   <si>
     <t>media.media_type</t>
@@ -995,7 +987,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1015,9 +1007,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1365,16 +1354,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC82330-B8C2-CD4B-8B66-6C9054D4C747}">
-  <dimension ref="A1:CJ7"/>
+  <dimension ref="A1:CI7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:88" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:87" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1390,19 +1379,19 @@
       <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5" t="s">
+        <v>3</v>
+      </c>
       <c r="K1" s="5" t="s">
         <v>3</v>
       </c>
@@ -1415,8 +1404,8 @@
       <c r="N1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="5" t="s">
-        <v>3</v>
+      <c r="O1" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="P1" s="6" t="s">
         <v>4</v>
@@ -1446,7 +1435,7 @@
         <v>4</v>
       </c>
       <c r="Y1" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Z1" s="6" t="s">
         <v>5</v>
@@ -1461,13 +1450,13 @@
         <v>5</v>
       </c>
       <c r="AD1" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AE1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="AF1" s="6" t="s">
         <v>7</v>
+      </c>
+      <c r="AF1" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="AG1" s="7" t="s">
         <v>8</v>
@@ -1505,8 +1494,8 @@
       <c r="AR1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="AS1" s="7" t="s">
-        <v>8</v>
+      <c r="AS1" s="8" t="s">
+        <v>9</v>
       </c>
       <c r="AT1" s="8" t="s">
         <v>9</v>
@@ -1514,8 +1503,8 @@
       <c r="AU1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="AV1" s="8" t="s">
-        <v>9</v>
+      <c r="AV1" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="AW1" s="9" t="s">
         <v>10</v>
@@ -1527,15 +1516,15 @@
         <v>10</v>
       </c>
       <c r="AZ1" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BA1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="BB1" s="9" t="s">
+      <c r="BB1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="BC1" s="29" t="s">
+      <c r="BC1" s="9" t="s">
         <v>11</v>
       </c>
       <c r="BD1" s="9" t="s">
@@ -1605,13 +1594,13 @@
         <v>11</v>
       </c>
       <c r="BZ1" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="CA1" s="9" t="s">
         <v>12</v>
       </c>
       <c r="CB1" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="CC1" s="9" t="s">
         <v>13</v>
@@ -1619,8 +1608,8 @@
       <c r="CD1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="CE1" s="9" t="s">
-        <v>13</v>
+      <c r="CE1" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="CF1" s="10" t="s">
         <v>14</v>
@@ -1632,13 +1621,10 @@
         <v>14</v>
       </c>
       <c r="CI1" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="CJ1" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
-    <row r="2" spans="1:88" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:87" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
@@ -1648,239 +1634,238 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>17</v>
       </c>
+      <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
+      <c r="O2" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="P2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="T2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="AC2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="AD2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AF2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AH2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AI2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AJ2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK2" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL2" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AM2" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="AN2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AO2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AP2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="AQ2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AR2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AS2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="AT2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="AU2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AV2" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AW2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="U2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="W2" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="X2" s="6" t="s">
+      <c r="AX2" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AY2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Y2" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="Z2" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="AA2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="AB2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="AC2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF2" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ2" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK2" s="7" t="s">
+      <c r="AZ2" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="BA2" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="BB2" s="28" t="s">
+        <v>243</v>
+      </c>
+      <c r="BC2" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD2" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE2" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH2" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI2" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ2" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL2" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM2" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN2" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO2" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ2" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR2" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS2" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT2" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU2" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV2" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW2" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX2" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY2" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA2" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC2" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD2" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE2" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="CF2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="CG2" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="CH2" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="AL2" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="AM2" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AN2" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="AO2" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="AP2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="AQ2" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="AR2" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="AS2" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AT2" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="AU2" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="AV2" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW2" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="AX2" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY2" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="AZ2" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="BA2" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="BB2" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="BC2" s="29" t="s">
-        <v>245</v>
-      </c>
-      <c r="BD2" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="BE2" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="BF2" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="BG2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="BH2" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="BI2" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="BJ2" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="BK2" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="BL2" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="BM2" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="BN2" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="BO2" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="BP2" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="BQ2" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="BR2" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="BS2" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="BT2" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="BU2" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="BV2" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="BW2" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="BX2" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="BY2" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="BZ2" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="CA2" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="CB2" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="CC2" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="CD2" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="CE2" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="CF2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="CG2" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="CH2" s="10" t="s">
-        <v>51</v>
-      </c>
       <c r="CI2" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="CJ2" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
-    <row r="3" spans="1:88" ht="139.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:87" ht="139.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>82</v>
       </c>
@@ -1893,62 +1878,62 @@
       <c r="D3" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="16" t="s">
+      <c r="E3" s="14"/>
+      <c r="F3" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="G3" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="I3" s="14"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17" t="s">
+      <c r="H3" s="14"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16" t="s">
         <v>88</v>
       </c>
+      <c r="K3" s="5"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="17" t="s">
+      <c r="M3" s="16" t="s">
         <v>89</v>
       </c>
+      <c r="N3" s="16" t="s">
+        <v>90</v>
+      </c>
       <c r="O3" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="P3" s="18" t="s">
         <v>91</v>
       </c>
+      <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="18" t="s">
+      <c r="R3" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="T3" s="18" t="s">
+      <c r="S3" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="U3" s="6"/>
-      <c r="V3" s="18" t="s">
+      <c r="T3" s="6"/>
+      <c r="U3" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="W3" s="18"/>
+      <c r="V3" s="17"/>
+      <c r="W3" s="6"/>
       <c r="X3" s="6"/>
-      <c r="Y3" s="6"/>
-      <c r="Z3" s="18" t="s">
+      <c r="Y3" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="AA3" s="18" t="s">
+      <c r="Z3" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="AB3" s="18" t="s">
+      <c r="AA3" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="AC3" s="18" t="s">
+      <c r="AB3" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="AD3" s="18" t="s">
+      <c r="AC3" s="17" t="s">
         <v>99</v>
       </c>
+      <c r="AD3" s="6"/>
       <c r="AE3" s="6"/>
-      <c r="AF3" s="6"/>
+      <c r="AF3" s="7"/>
       <c r="AG3" s="7"/>
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
@@ -1960,115 +1945,114 @@
       <c r="AO3" s="7"/>
       <c r="AP3" s="7"/>
       <c r="AQ3" s="7"/>
-      <c r="AR3" s="7"/>
-      <c r="AS3" s="7" t="s">
+      <c r="AR3" s="7" t="s">
         <v>100</v>
       </c>
+      <c r="AS3" s="8"/>
       <c r="AT3" s="8"/>
       <c r="AU3" s="8"/>
-      <c r="AV3" s="8"/>
+      <c r="AV3" s="9"/>
       <c r="AW3" s="9"/>
-      <c r="AX3" s="9"/>
-      <c r="AY3" s="19" t="s">
+      <c r="AX3" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="AZ3" s="19"/>
-      <c r="BA3" s="20" t="s">
+      <c r="AY3" s="18"/>
+      <c r="AZ3" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="BB3" s="20" t="s">
+      <c r="BA3" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="BC3" s="30"/>
-      <c r="BD3" s="20" t="s">
+      <c r="BB3" s="29"/>
+      <c r="BC3" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="BE3" s="20" t="s">
+      <c r="BD3" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="BF3" s="20" t="s">
+      <c r="BE3" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="BG3" s="20" t="s">
+      <c r="BF3" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="BH3" s="20" t="s">
+      <c r="BG3" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="BI3" s="20" t="s">
+      <c r="BH3" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="BJ3" s="20" t="s">
+      <c r="BI3" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="BK3" s="20" t="s">
+      <c r="BJ3" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="BL3" s="19" t="s">
+      <c r="BK3" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="BM3" s="19"/>
-      <c r="BN3" s="19" t="s">
+      <c r="BL3" s="18"/>
+      <c r="BM3" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="BO3" s="21" t="s">
+      <c r="BN3" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="BP3" s="21" t="s">
+      <c r="BO3" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="BQ3" s="21" t="s">
+      <c r="BP3" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="BR3" s="21" t="s">
+      <c r="BQ3" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="BS3" s="19" t="s">
+      <c r="BR3" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="BT3" s="19" t="s">
+      <c r="BS3" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="BU3" s="19" t="s">
+      <c r="BT3" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="BV3" s="19" t="s">
+      <c r="BU3" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="BW3" s="19" t="s">
+      <c r="BV3" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="BX3" s="19" t="s">
+      <c r="BW3" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="BY3" s="19" t="s">
+      <c r="BX3" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="BZ3" s="20"/>
-      <c r="CA3" s="19" t="s">
+      <c r="BY3" s="19"/>
+      <c r="BZ3" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="CB3" s="19" t="s">
+      <c r="CA3" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="CC3" s="19" t="s">
+      <c r="CB3" s="18" t="s">
         <v>127</v>
       </c>
+      <c r="CC3" s="18" t="s">
+        <v>127</v>
+      </c>
       <c r="CD3" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="CE3" s="20" t="s">
         <v>128</v>
       </c>
+      <c r="CE3" s="10"/>
       <c r="CF3" s="10"/>
       <c r="CG3" s="10"/>
       <c r="CH3" s="10"/>
-      <c r="CI3" s="10"/>
-      <c r="CJ3" s="10" t="s">
-        <v>244</v>
+      <c r="CI3" s="10" t="s">
+        <v>242</v>
       </c>
     </row>
-    <row r="4" spans="1:88" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:87" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>129</v>
       </c>
@@ -2082,16 +2066,16 @@
       <c r="E4" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>131</v>
-      </c>
+      <c r="G4" s="3"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="I4" s="5"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="K4" s="5" t="s">
+        <v>132</v>
+      </c>
       <c r="L4" s="5" t="s">
         <v>132</v>
       </c>
@@ -2101,12 +2085,10 @@
       <c r="N4" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="O4" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>132</v>
-      </c>
+      <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
@@ -2115,20 +2097,20 @@
       <c r="V4" s="6"/>
       <c r="W4" s="6"/>
       <c r="X4" s="6"/>
-      <c r="Y4" s="6"/>
+      <c r="Y4" s="6" t="s">
+        <v>133</v>
+      </c>
       <c r="Z4" s="6" t="s">
         <v>133</v>
       </c>
       <c r="AA4" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="AB4" s="6" t="s">
-        <v>133</v>
-      </c>
+      <c r="AB4" s="6"/>
       <c r="AC4" s="6"/>
       <c r="AD4" s="6"/>
       <c r="AE4" s="6"/>
-      <c r="AF4" s="6"/>
+      <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
@@ -2141,17 +2123,17 @@
       <c r="AP4" s="7"/>
       <c r="AQ4" s="7"/>
       <c r="AR4" s="7"/>
-      <c r="AS4" s="7"/>
+      <c r="AS4" s="8"/>
       <c r="AT4" s="8"/>
       <c r="AU4" s="8"/>
-      <c r="AV4" s="8"/>
+      <c r="AV4" s="9"/>
       <c r="AW4" s="9"/>
       <c r="AX4" s="9"/>
       <c r="AY4" s="9"/>
       <c r="AZ4" s="9"/>
       <c r="BA4" s="9"/>
-      <c r="BB4" s="9"/>
-      <c r="BC4" s="29"/>
+      <c r="BB4" s="28"/>
+      <c r="BC4" s="9"/>
       <c r="BD4" s="9"/>
       <c r="BE4" s="9"/>
       <c r="BF4" s="9"/>
@@ -2179,16 +2161,15 @@
       <c r="CB4" s="9"/>
       <c r="CC4" s="9"/>
       <c r="CD4" s="9"/>
-      <c r="CE4" s="9"/>
+      <c r="CE4" s="10"/>
       <c r="CF4" s="10"/>
       <c r="CG4" s="10"/>
       <c r="CH4" s="10"/>
-      <c r="CI4" s="10"/>
-      <c r="CJ4" s="10" t="s">
-        <v>244</v>
+      <c r="CI4" s="10" t="s">
+        <v>242</v>
       </c>
     </row>
-    <row r="5" spans="1:88" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:87" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>134</v>
       </c>
@@ -2204,44 +2185,44 @@
       <c r="E5" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="K5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="L5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="Q5" s="6" t="s">
-        <v>136</v>
-      </c>
       <c r="R5" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="S5" s="6" t="s">
         <v>136</v>
@@ -2256,13 +2237,13 @@
         <v>136</v>
       </c>
       <c r="W5" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="X5" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="Y5" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="Z5" s="6" t="s">
         <v>139</v>
@@ -2274,7 +2255,7 @@
         <v>139</v>
       </c>
       <c r="AC5" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="AD5" s="6" t="s">
         <v>137</v>
@@ -2282,179 +2263,176 @@
       <c r="AE5" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="AF5" s="6" t="s">
-        <v>137</v>
+      <c r="AF5" s="7" t="s">
+        <v>136</v>
       </c>
       <c r="AG5" s="7" t="s">
         <v>136</v>
       </c>
       <c r="AH5" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="AI5" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AJ5" s="7" t="s">
         <v>136</v>
       </c>
       <c r="AK5" s="7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="AL5" s="7" t="s">
         <v>139</v>
       </c>
       <c r="AM5" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="AN5" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="AO5" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="AP5" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="AQ5" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="AR5" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="AS5" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="AT5" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="AU5" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="AV5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="AW5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="AX5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="AY5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="AZ5" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="AN5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AO5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AP5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AQ5" s="7" t="s">
+      <c r="BA5" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="AR5" s="7" t="s">
+      <c r="BB5" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="AS5" s="7" t="s">
+      <c r="BC5" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="AT5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="AU5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="AV5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="AW5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="AX5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="AY5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="AZ5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="BA5" s="22" t="s">
+      <c r="BD5" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="BE5" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="BB5" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="BC5" s="31" t="s">
+      <c r="BF5" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="BG5" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="BH5" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="BI5" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="BJ5" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="BK5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="BL5" s="9" t="s">
         <v>137</v>
-      </c>
-      <c r="BD5" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="BE5" s="22" t="s">
-        <v>136</v>
-      </c>
-      <c r="BF5" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="BG5" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="BH5" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="BI5" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="BJ5" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="BK5" s="22" t="s">
-        <v>136</v>
-      </c>
-      <c r="BL5" s="9" t="s">
-        <v>136</v>
       </c>
       <c r="BM5" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="BN5" s="9" t="s">
+      <c r="BN5" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="BO5" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP5" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="BQ5" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="BR5" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="BO5" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="BP5" s="23" t="s">
+      <c r="BS5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="BT5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="BU5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="BV5" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="BQ5" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="BR5" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="BS5" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="BT5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="BU5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="BV5" s="9" t="s">
-        <v>136</v>
-      </c>
       <c r="BW5" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="BX5" s="9" t="s">
         <v>140</v>
       </c>
       <c r="BY5" s="9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="BZ5" s="9" t="s">
         <v>137</v>
       </c>
       <c r="CA5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="CB5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="CC5" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="CD5" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="CB5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="CC5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="CD5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="CE5" s="9" t="s">
-        <v>137</v>
+      <c r="CE5" s="10" t="s">
+        <v>136</v>
       </c>
       <c r="CF5" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="CG5" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="CH5" s="10" t="s">
         <v>136</v>
       </c>
       <c r="CI5" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="CJ5" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
-    <row r="6" spans="1:88" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:87" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>142</v>
       </c>
@@ -2466,25 +2444,23 @@
       <c r="E6" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>146</v>
-      </c>
+      <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
+      <c r="O6" s="6"/>
       <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6" t="s">
-        <v>147</v>
-      </c>
+      <c r="Q6" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="R6" s="6"/>
       <c r="S6" s="6"/>
       <c r="T6" s="6"/>
       <c r="U6" s="6"/>
@@ -2495,16 +2471,16 @@
       <c r="Z6" s="6"/>
       <c r="AA6" s="6"/>
       <c r="AB6" s="6"/>
-      <c r="AC6" s="6"/>
+      <c r="AC6" s="6" t="s">
+        <v>147</v>
+      </c>
       <c r="AD6" s="6" t="s">
         <v>148</v>
       </c>
       <c r="AE6" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="AF6" s="6" t="s">
-        <v>150</v>
-      </c>
+      <c r="AF6" s="7"/>
       <c r="AG6" s="7"/>
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
@@ -2515,23 +2491,23 @@
       <c r="AN6" s="7"/>
       <c r="AO6" s="7"/>
       <c r="AP6" s="7"/>
-      <c r="AQ6" s="7"/>
-      <c r="AR6" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="AS6" s="7"/>
+      <c r="AQ6" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="AR6" s="7"/>
+      <c r="AS6" s="8"/>
       <c r="AT6" s="8"/>
       <c r="AU6" s="8"/>
-      <c r="AV6" s="8"/>
+      <c r="AV6" s="9"/>
       <c r="AW6" s="9"/>
       <c r="AX6" s="9"/>
       <c r="AY6" s="9"/>
       <c r="AZ6" s="9"/>
       <c r="BA6" s="9"/>
-      <c r="BB6" s="9"/>
-      <c r="BC6" s="31" t="s">
-        <v>246</v>
-      </c>
+      <c r="BB6" s="30" t="s">
+        <v>244</v>
+      </c>
+      <c r="BC6" s="9"/>
       <c r="BD6" s="9"/>
       <c r="BE6" s="9"/>
       <c r="BF6" s="9"/>
@@ -2540,310 +2516,306 @@
       <c r="BI6" s="9"/>
       <c r="BJ6" s="9"/>
       <c r="BK6" s="9"/>
-      <c r="BL6" s="9"/>
+      <c r="BL6" s="9" t="s">
+        <v>151</v>
+      </c>
       <c r="BM6" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="BN6" s="9" t="s">
-        <v>153</v>
-      </c>
+      <c r="BN6" s="9"/>
       <c r="BO6" s="9"/>
       <c r="BP6" s="9"/>
       <c r="BQ6" s="9"/>
-      <c r="BR6" s="9"/>
-      <c r="BS6" s="9" t="s">
-        <v>154</v>
-      </c>
+      <c r="BR6" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="BS6" s="9"/>
       <c r="BT6" s="9"/>
       <c r="BU6" s="9"/>
       <c r="BV6" s="9"/>
       <c r="BW6" s="9"/>
       <c r="BX6" s="9"/>
-      <c r="BY6" s="9"/>
+      <c r="BY6" s="9" t="s">
+        <v>154</v>
+      </c>
       <c r="BZ6" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="CA6" s="9" t="s">
-        <v>156</v>
-      </c>
+      <c r="CA6" s="9"/>
       <c r="CB6" s="9"/>
       <c r="CC6" s="9"/>
-      <c r="CD6" s="9"/>
-      <c r="CE6" s="9" t="s">
-        <v>157</v>
-      </c>
+      <c r="CD6" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="CE6" s="10"/>
       <c r="CF6" s="10"/>
       <c r="CG6" s="10"/>
       <c r="CH6" s="10"/>
-      <c r="CI6" s="10"/>
-      <c r="CJ6" s="10" t="s">
-        <v>244</v>
+      <c r="CI6" s="10" t="s">
+        <v>242</v>
       </c>
     </row>
-    <row r="7" spans="1:88" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:87" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="J7" s="24" t="s">
+      <c r="K7" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L7" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="M7" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="N7" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="O7" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="P7" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="P7" s="25" t="s">
+      <c r="Q7" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="Q7" s="25" t="s">
+      <c r="R7" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="R7" s="25" t="s">
+      <c r="S7" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="S7" s="6" t="s">
+      <c r="T7" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="T7" s="6" t="s">
+      <c r="U7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="U7" s="6" t="s">
+      <c r="V7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="V7" s="6" t="s">
+      <c r="W7" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="W7" s="6" t="s">
+      <c r="X7" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="X7" s="6" t="s">
+      <c r="Y7" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="Y7" s="6" t="s">
+      <c r="Z7" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="Z7" s="25" t="s">
+      <c r="AA7" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="AA7" s="25" t="s">
+      <c r="AB7" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="AB7" s="25" t="s">
+      <c r="AC7" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="AC7" s="6" t="s">
+      <c r="AD7" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="AD7" s="6" t="s">
+      <c r="AE7" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="AE7" s="25" t="s">
+      <c r="AF7" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="AF7" s="6" t="s">
+      <c r="AG7" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="AG7" s="26" t="s">
+      <c r="AH7" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="AH7" s="26" t="s">
+      <c r="AI7" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="AI7" s="26" t="s">
+      <c r="AJ7" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="AJ7" s="26" t="s">
+      <c r="AK7" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="AK7" s="26" t="s">
+      <c r="AL7" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="AL7" s="26" t="s">
+      <c r="AM7" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="AM7" s="26" t="s">
+      <c r="AN7" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="AN7" s="26" t="s">
+      <c r="AO7" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="AO7" s="26" t="s">
+      <c r="AP7" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="AP7" s="26" t="s">
+      <c r="AQ7" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="AQ7" s="26" t="s">
+      <c r="AR7" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="AR7" s="26" t="s">
+      <c r="AS7" s="26" t="s">
         <v>201</v>
       </c>
-      <c r="AS7" s="26" t="s">
+      <c r="AT7" s="26" t="s">
         <v>202</v>
       </c>
-      <c r="AT7" s="27" t="s">
+      <c r="AU7" s="26" t="s">
         <v>203</v>
       </c>
-      <c r="AU7" s="27" t="s">
+      <c r="AV7" s="26" t="s">
         <v>204</v>
       </c>
-      <c r="AV7" s="27" t="s">
+      <c r="AW7" s="26" t="s">
         <v>205</v>
       </c>
-      <c r="AW7" s="27" t="s">
+      <c r="AX7" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="AX7" s="27" t="s">
+      <c r="AY7" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="AY7" s="9" t="s">
+      <c r="AZ7" s="26" t="s">
         <v>208</v>
       </c>
-      <c r="AZ7" s="9" t="s">
+      <c r="BA7" s="26" t="s">
         <v>209</v>
       </c>
-      <c r="BA7" s="27" t="s">
+      <c r="BB7" s="31" t="s">
+        <v>245</v>
+      </c>
+      <c r="BC7" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="BB7" s="27" t="s">
+      <c r="BD7" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="BC7" s="32" t="s">
-        <v>247</v>
-      </c>
-      <c r="BD7" s="27" t="s">
+      <c r="BE7" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="BE7" s="9" t="s">
+      <c r="BF7" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="BF7" s="27" t="s">
+      <c r="BG7" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="BG7" s="27" t="s">
+      <c r="BH7" s="26" t="s">
         <v>215</v>
       </c>
-      <c r="BH7" s="27" t="s">
+      <c r="BI7" s="26" t="s">
         <v>216</v>
       </c>
-      <c r="BI7" s="27" t="s">
+      <c r="BJ7" s="26" t="s">
         <v>217</v>
       </c>
-      <c r="BJ7" s="27" t="s">
+      <c r="BK7" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="BK7" s="27" t="s">
+      <c r="BL7" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="BL7" s="9" t="s">
+      <c r="BM7" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="BM7" s="9" t="s">
+      <c r="BN7" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="BN7" s="9" t="s">
+      <c r="BO7" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="BO7" s="9" t="s">
+      <c r="BP7" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="BP7" s="9" t="s">
+      <c r="BQ7" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="BQ7" s="9" t="s">
+      <c r="BR7" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="BR7" s="9" t="s">
+      <c r="BS7" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="BS7" s="9" t="s">
+      <c r="BT7" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="BT7" s="9" t="s">
+      <c r="BU7" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="BU7" s="9" t="s">
+      <c r="BV7" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="BV7" s="9" t="s">
+      <c r="BW7" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="BW7" s="9" t="s">
+      <c r="BX7" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="BX7" s="9" t="s">
+      <c r="BY7" s="27" t="s">
         <v>232</v>
       </c>
-      <c r="BY7" s="9" t="s">
+      <c r="BZ7" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="BZ7" s="28" t="s">
+      <c r="CA7" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="CA7" s="9" t="s">
+      <c r="CB7" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="CB7" s="9" t="s">
+      <c r="CC7" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="CC7" s="9" t="s">
+      <c r="CD7" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="CD7" s="9" t="s">
+      <c r="CE7" s="26" t="s">
         <v>238</v>
       </c>
-      <c r="CE7" s="9" t="s">
+      <c r="CF7" s="26" t="s">
         <v>239</v>
       </c>
-      <c r="CF7" s="27" t="s">
+      <c r="CG7" s="26" t="s">
         <v>240</v>
       </c>
-      <c r="CG7" s="27" t="s">
+      <c r="CH7" s="26" t="s">
         <v>241</v>
       </c>
-      <c r="CH7" s="27" t="s">
+      <c r="CI7" s="10" t="s">
         <v>242</v>
-      </c>
-      <c r="CI7" s="27" t="s">
-        <v>243</v>
-      </c>
-      <c r="CJ7" s="10" t="s">
-        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated tests and test ingest files
</commit_message>
<xml_diff>
--- a/spec/fixtures/batch_submission_manifest_errors_columns.xlsx
+++ b/spec/fixtures/batch_submission_manifest_errors_columns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource_SF/spec/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smc101/vagrant/morphosource-vagrant/MorphoSource/spec/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3896FF05-6D15-A947-AE64-F70F7D1ED464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5EF912-C8FF-6949-B681-DBE5E924719B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2380" yWindow="1000" windowWidth="27640" windowHeight="15740" xr2:uid="{B67D321E-7C1E-1B4C-B0D3-48C3E7F2330E}"/>
+    <workbookView xWindow="2380" yWindow="980" windowWidth="27640" windowHeight="15740" xr2:uid="{B67D321E-7C1E-1B4C-B0D3-48C3E7F2330E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="244">
   <si>
     <t>Field Section</t>
   </si>
@@ -299,9 +299,6 @@
   </si>
   <si>
     <t>Ignore this in most use cases! Parent media filename OR URL endpoint link for downloading parent media file</t>
-  </si>
-  <si>
-    <t>iDigBio UUID for specimen record</t>
   </si>
   <si>
     <t>Collection code modifier (e.g., "VP-", typically designates a sub-collection within a repository. Not a universal element because not all repositories have sub-collections. However, this field is critical when applicable to avoid confusing specimens from different sub-collections. Please make sure you do not incorrectly omit a collection code fromt the specimen identifier</t>
@@ -601,9 +598,6 @@
   </si>
   <si>
     <t>biological_specimen.ms_id</t>
-  </si>
-  <si>
-    <t>biological_specimen.idigbio_uuid</t>
   </si>
   <si>
     <t>biological_specimen.occurrence_id</t>
@@ -1058,9 +1052,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1098,7 +1092,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1204,7 +1198,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1346,7 +1340,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1354,7 +1348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC82330-B8C2-CD4B-8B66-6C9054D4C747}">
-  <dimension ref="A1:CI7"/>
+  <dimension ref="A1:CH7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
@@ -1363,7 +1357,7 @@
     <col min="9" max="9" width="23.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:87" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:86" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1401,8 +1395,8 @@
       <c r="M1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>3</v>
+      <c r="N1" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>4</v>
@@ -1432,7 +1426,7 @@
         <v>4</v>
       </c>
       <c r="X1" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Y1" s="6" t="s">
         <v>5</v>
@@ -1447,13 +1441,13 @@
         <v>5</v>
       </c>
       <c r="AC1" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AD1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="AE1" s="6" t="s">
         <v>7</v>
+      </c>
+      <c r="AE1" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="AF1" s="7" t="s">
         <v>8</v>
@@ -1491,8 +1485,8 @@
       <c r="AQ1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="AR1" s="7" t="s">
-        <v>8</v>
+      <c r="AR1" s="8" t="s">
+        <v>9</v>
       </c>
       <c r="AS1" s="8" t="s">
         <v>9</v>
@@ -1500,8 +1494,8 @@
       <c r="AT1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="AU1" s="8" t="s">
-        <v>9</v>
+      <c r="AU1" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="AV1" s="9" t="s">
         <v>10</v>
@@ -1513,15 +1507,15 @@
         <v>10</v>
       </c>
       <c r="AY1" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AZ1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="BA1" s="9" t="s">
+      <c r="BA1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="BB1" s="28" t="s">
+      <c r="BB1" s="9" t="s">
         <v>11</v>
       </c>
       <c r="BC1" s="9" t="s">
@@ -1591,13 +1585,13 @@
         <v>11</v>
       </c>
       <c r="BY1" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="BZ1" s="9" t="s">
         <v>12</v>
       </c>
       <c r="CA1" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="CB1" s="9" t="s">
         <v>13</v>
@@ -1605,8 +1599,8 @@
       <c r="CC1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="CD1" s="9" t="s">
-        <v>13</v>
+      <c r="CD1" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="CE1" s="10" t="s">
         <v>14</v>
@@ -1618,13 +1612,10 @@
         <v>14</v>
       </c>
       <c r="CH1" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="CI1" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
-    <row r="2" spans="1:87" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:86" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
@@ -1644,228 +1635,227 @@
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="N2" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="W2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="X2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y2" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z2" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AH2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AJ2" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AK2" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="AL2" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="AM2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO2" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="AP2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AQ2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AR2" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="AS2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="AT2" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU2" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AV2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="T2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="W2" s="6" t="s">
+      <c r="AW2" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AX2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="X2" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y2" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="Z2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD2" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE2" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="AF2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="AH2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="AI2" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="AJ2" s="7" t="s">
+      <c r="AY2" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ2" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="BA2" s="28" t="s">
+        <v>241</v>
+      </c>
+      <c r="BB2" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="BC2" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="BD2" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="BE2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="BF2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="BG2" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="BH2" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="BI2" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="BJ2" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="BK2" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="BL2" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="BM2" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="BN2" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="BO2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="BP2" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="BQ2" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR2" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="BS2" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="BT2" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="BU2" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="BV2" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="BW2" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="BX2" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="BY2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="BZ2" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="CA2" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="CB2" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="CC2" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="CD2" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="CE2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="CF2" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="CG2" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="AK2" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="AL2" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AM2" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="AN2" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="AP2" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="AQ2" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="AR2" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AS2" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="AT2" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="AU2" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="AV2" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="AW2" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="AX2" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="AY2" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="AZ2" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="BA2" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="BB2" s="28" t="s">
-        <v>243</v>
-      </c>
-      <c r="BC2" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="BD2" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="BE2" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="BF2" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="BG2" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="BH2" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="BI2" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="BJ2" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="BK2" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="BL2" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="BM2" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="BN2" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="BO2" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="BP2" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="BQ2" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="BR2" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="BS2" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="BT2" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="BU2" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="BV2" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="BW2" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="BX2" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="BY2" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="BZ2" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="CA2" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="CB2" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="CC2" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="CD2" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="CE2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="CF2" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="CG2" s="10" t="s">
-        <v>51</v>
-      </c>
       <c r="CH2" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="CI2" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
-    <row r="3" spans="1:87" ht="139.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:86" ht="139.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>82</v>
       </c>
@@ -1887,35 +1877,35 @@
       </c>
       <c r="H3" s="14"/>
       <c r="I3" s="16"/>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
       <c r="M3" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="N3" s="16" t="s">
+      <c r="N3" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="O3" s="17" t="s">
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
       <c r="R3" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="S3" s="17" t="s">
+      <c r="S3" s="6"/>
+      <c r="T3" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="T3" s="6"/>
-      <c r="U3" s="17" t="s">
+      <c r="U3" s="17"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="V3" s="17"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
       <c r="Y3" s="17" t="s">
         <v>95</v>
       </c>
@@ -1928,11 +1918,9 @@
       <c r="AB3" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="AC3" s="17" t="s">
-        <v>99</v>
-      </c>
+      <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
-      <c r="AE3" s="6"/>
+      <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
       <c r="AG3" s="7"/>
       <c r="AH3" s="7"/>
@@ -1944,26 +1932,28 @@
       <c r="AN3" s="7"/>
       <c r="AO3" s="7"/>
       <c r="AP3" s="7"/>
-      <c r="AQ3" s="7"/>
-      <c r="AR3" s="7" t="s">
-        <v>100</v>
-      </c>
+      <c r="AQ3" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR3" s="8"/>
       <c r="AS3" s="8"/>
       <c r="AT3" s="8"/>
-      <c r="AU3" s="8"/>
+      <c r="AU3" s="9"/>
       <c r="AV3" s="9"/>
-      <c r="AW3" s="9"/>
-      <c r="AX3" s="18" t="s">
+      <c r="AW3" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="AX3" s="18"/>
+      <c r="AY3" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="AY3" s="18"/>
       <c r="AZ3" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="BA3" s="19" t="s">
+      <c r="BA3" s="29"/>
+      <c r="BB3" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="BB3" s="29"/>
       <c r="BC3" s="19" t="s">
         <v>104</v>
       </c>
@@ -1985,14 +1975,14 @@
       <c r="BI3" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="BJ3" s="19" t="s">
+      <c r="BJ3" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="BK3" s="18" t="s">
+      <c r="BK3" s="18"/>
+      <c r="BL3" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="BL3" s="18"/>
-      <c r="BM3" s="18" t="s">
+      <c r="BM3" s="20" t="s">
         <v>113</v>
       </c>
       <c r="BN3" s="20" t="s">
@@ -2004,7 +1994,7 @@
       <c r="BP3" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="BQ3" s="20" t="s">
+      <c r="BQ3" s="18" t="s">
         <v>117</v>
       </c>
       <c r="BR3" s="18" t="s">
@@ -2025,10 +2015,10 @@
       <c r="BW3" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="BX3" s="18" t="s">
+      <c r="BX3" s="19"/>
+      <c r="BY3" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="BY3" s="19"/>
       <c r="BZ3" s="18" t="s">
         <v>125</v>
       </c>
@@ -2036,58 +2026,55 @@
         <v>126</v>
       </c>
       <c r="CB3" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="CC3" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="CC3" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="CD3" s="19" t="s">
-        <v>128</v>
-      </c>
+      <c r="CD3" s="10"/>
       <c r="CE3" s="10"/>
       <c r="CF3" s="10"/>
       <c r="CG3" s="10"/>
-      <c r="CH3" s="10"/>
-      <c r="CI3" s="10" t="s">
-        <v>242</v>
+      <c r="CH3" s="10" t="s">
+        <v>240</v>
       </c>
     </row>
-    <row r="4" spans="1:87" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:86" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
+      <c r="J4" s="5" t="s">
+        <v>131</v>
+      </c>
       <c r="K4" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>132</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
@@ -2096,20 +2083,20 @@
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
       <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
+      <c r="X4" s="6" t="s">
+        <v>132</v>
+      </c>
       <c r="Y4" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="AA4" s="6" t="s">
-        <v>133</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="AA4" s="6"/>
       <c r="AB4" s="6"/>
       <c r="AC4" s="6"/>
       <c r="AD4" s="6"/>
-      <c r="AE4" s="6"/>
+      <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
@@ -2122,17 +2109,17 @@
       <c r="AO4" s="7"/>
       <c r="AP4" s="7"/>
       <c r="AQ4" s="7"/>
-      <c r="AR4" s="7"/>
+      <c r="AR4" s="8"/>
       <c r="AS4" s="8"/>
       <c r="AT4" s="8"/>
-      <c r="AU4" s="8"/>
+      <c r="AU4" s="9"/>
       <c r="AV4" s="9"/>
       <c r="AW4" s="9"/>
       <c r="AX4" s="9"/>
       <c r="AY4" s="9"/>
       <c r="AZ4" s="9"/>
-      <c r="BA4" s="9"/>
-      <c r="BB4" s="28"/>
+      <c r="BA4" s="28"/>
+      <c r="BB4" s="9"/>
       <c r="BC4" s="9"/>
       <c r="BD4" s="9"/>
       <c r="BE4" s="9"/>
@@ -2160,292 +2147,288 @@
       <c r="CA4" s="9"/>
       <c r="CB4" s="9"/>
       <c r="CC4" s="9"/>
-      <c r="CD4" s="9"/>
+      <c r="CD4" s="10"/>
       <c r="CE4" s="10"/>
       <c r="CF4" s="10"/>
       <c r="CG4" s="10"/>
-      <c r="CH4" s="10"/>
-      <c r="CI4" s="10" t="s">
-        <v>242</v>
+      <c r="CH4" s="10" t="s">
+        <v>240</v>
       </c>
     </row>
-    <row r="5" spans="1:87" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:86" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>135</v>
-      </c>
       <c r="C5" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>137</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>135</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P5" s="6" t="s">
         <v>136</v>
       </c>
       <c r="Q5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="U5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="V5" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="W5" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="X5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="Z5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="AA5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="AB5" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="S5" s="6" t="s">
+      <c r="AC5" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="T5" s="6" t="s">
+      <c r="AD5" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="U5" s="6" t="s">
+      <c r="AE5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AF5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG5" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="AH5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AI5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AJ5" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AK5" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="AL5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AM5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AN5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="AO5" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="AP5" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="V5" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="W5" s="6" t="s">
+      <c r="AQ5" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="AR5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="AT5" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="AU5" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="AV5" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="AW5" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="AX5" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="AY5" s="21" t="s">
         <v>138</v>
-      </c>
-      <c r="X5" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="Y5" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="Z5" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="AA5" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="AB5" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="AC5" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="AD5" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="AE5" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="AF5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AG5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AH5" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="AI5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AJ5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AK5" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="AL5" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="AM5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AN5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AO5" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AP5" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="AQ5" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="AR5" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="AS5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="AT5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="AU5" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="AV5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="AW5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="AX5" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="AY5" s="9" t="s">
-        <v>136</v>
       </c>
       <c r="AZ5" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="BA5" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="BB5" s="30" t="s">
-        <v>137</v>
+      <c r="BA5" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="BB5" s="21" t="s">
+        <v>139</v>
       </c>
       <c r="BC5" s="21" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="BD5" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="BE5" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="BF5" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="BG5" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="BH5" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="BI5" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="BJ5" s="21" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="BJ5" s="9" t="s">
+        <v>135</v>
       </c>
       <c r="BK5" s="9" t="s">
         <v>136</v>
       </c>
       <c r="BL5" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="BM5" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="BM5" s="22" t="s">
+        <v>140</v>
       </c>
       <c r="BN5" s="22" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="BO5" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="BP5" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="BQ5" s="22" t="s">
-        <v>139</v>
+        <v>138</v>
+      </c>
+      <c r="BQ5" s="9" t="s">
+        <v>136</v>
       </c>
       <c r="BR5" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="BS5" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="BT5" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="BU5" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="BV5" s="9" t="s">
         <v>139</v>
       </c>
       <c r="BW5" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="BX5" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="BY5" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="BZ5" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="CA5" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="CB5" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="CC5" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="CD5" s="9" t="s">
+      <c r="CD5" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="CE5" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="CE5" s="10" t="s">
-        <v>136</v>
-      </c>
       <c r="CF5" s="10" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="CG5" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="CH5" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="CI5" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
-    <row r="6" spans="1:87" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:86" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>144</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>145</v>
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
@@ -2454,12 +2437,12 @@
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
+      <c r="N6" s="6"/>
       <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6" t="s">
-        <v>146</v>
-      </c>
+      <c r="P6" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
       <c r="T6" s="6"/>
@@ -2470,16 +2453,16 @@
       <c r="Y6" s="6"/>
       <c r="Z6" s="6"/>
       <c r="AA6" s="6"/>
-      <c r="AB6" s="6"/>
+      <c r="AB6" s="6" t="s">
+        <v>146</v>
+      </c>
       <c r="AC6" s="6" t="s">
         <v>147</v>
       </c>
       <c r="AD6" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="AE6" s="6" t="s">
-        <v>149</v>
-      </c>
+      <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
       <c r="AG6" s="7"/>
       <c r="AH6" s="7"/>
@@ -2490,23 +2473,23 @@
       <c r="AM6" s="7"/>
       <c r="AN6" s="7"/>
       <c r="AO6" s="7"/>
-      <c r="AP6" s="7"/>
-      <c r="AQ6" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="AR6" s="7"/>
+      <c r="AP6" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="AQ6" s="7"/>
+      <c r="AR6" s="8"/>
       <c r="AS6" s="8"/>
       <c r="AT6" s="8"/>
-      <c r="AU6" s="8"/>
+      <c r="AU6" s="9"/>
       <c r="AV6" s="9"/>
       <c r="AW6" s="9"/>
       <c r="AX6" s="9"/>
       <c r="AY6" s="9"/>
       <c r="AZ6" s="9"/>
-      <c r="BA6" s="9"/>
-      <c r="BB6" s="30" t="s">
-        <v>244</v>
-      </c>
+      <c r="BA6" s="30" t="s">
+        <v>242</v>
+      </c>
+      <c r="BB6" s="9"/>
       <c r="BC6" s="9"/>
       <c r="BD6" s="9"/>
       <c r="BE6" s="9"/>
@@ -2515,307 +2498,303 @@
       <c r="BH6" s="9"/>
       <c r="BI6" s="9"/>
       <c r="BJ6" s="9"/>
-      <c r="BK6" s="9"/>
+      <c r="BK6" s="9" t="s">
+        <v>150</v>
+      </c>
       <c r="BL6" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="BM6" s="9" t="s">
-        <v>152</v>
-      </c>
+      <c r="BM6" s="9"/>
       <c r="BN6" s="9"/>
       <c r="BO6" s="9"/>
       <c r="BP6" s="9"/>
-      <c r="BQ6" s="9"/>
-      <c r="BR6" s="9" t="s">
-        <v>153</v>
-      </c>
+      <c r="BQ6" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="BR6" s="9"/>
       <c r="BS6" s="9"/>
       <c r="BT6" s="9"/>
       <c r="BU6" s="9"/>
       <c r="BV6" s="9"/>
       <c r="BW6" s="9"/>
-      <c r="BX6" s="9"/>
+      <c r="BX6" s="9" t="s">
+        <v>153</v>
+      </c>
       <c r="BY6" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="BZ6" s="9" t="s">
-        <v>155</v>
-      </c>
+      <c r="BZ6" s="9"/>
       <c r="CA6" s="9"/>
       <c r="CB6" s="9"/>
-      <c r="CC6" s="9"/>
-      <c r="CD6" s="9" t="s">
-        <v>156</v>
-      </c>
+      <c r="CC6" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="CD6" s="10"/>
       <c r="CE6" s="10"/>
       <c r="CF6" s="10"/>
       <c r="CG6" s="10"/>
-      <c r="CH6" s="10"/>
-      <c r="CI6" s="10" t="s">
-        <v>242</v>
+      <c r="CH6" s="10" t="s">
+        <v>240</v>
       </c>
     </row>
-    <row r="7" spans="1:87" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:86" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="J7" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="K7" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L7" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="M7" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="N7" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="O7" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="O7" s="24" t="s">
+      <c r="P7" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="P7" s="24" t="s">
+      <c r="Q7" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="Q7" s="24" t="s">
+      <c r="R7" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="R7" s="6" t="s">
+      <c r="S7" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="S7" s="6" t="s">
+      <c r="T7" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="T7" s="6" t="s">
+      <c r="U7" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="U7" s="6" t="s">
+      <c r="V7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="V7" s="6" t="s">
+      <c r="W7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="W7" s="6" t="s">
+      <c r="X7" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="X7" s="6" t="s">
+      <c r="Y7" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="Y7" s="24" t="s">
+      <c r="Z7" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="Z7" s="24" t="s">
+      <c r="AA7" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="AA7" s="24" t="s">
+      <c r="AB7" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="AB7" s="6" t="s">
+      <c r="AC7" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="AC7" s="6" t="s">
+      <c r="AD7" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="AD7" s="24" t="s">
+      <c r="AE7" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="AE7" s="6" t="s">
+      <c r="AF7" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="AF7" s="25" t="s">
+      <c r="AG7" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="AG7" s="25" t="s">
+      <c r="AH7" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="AH7" s="25" t="s">
+      <c r="AI7" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="AI7" s="25" t="s">
+      <c r="AJ7" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="AJ7" s="25" t="s">
+      <c r="AK7" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="AK7" s="25" t="s">
+      <c r="AL7" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="AL7" s="25" t="s">
+      <c r="AM7" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="AM7" s="25" t="s">
+      <c r="AN7" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="AN7" s="25" t="s">
+      <c r="AO7" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="AO7" s="25" t="s">
+      <c r="AP7" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="AP7" s="25" t="s">
+      <c r="AQ7" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="AQ7" s="25" t="s">
+      <c r="AR7" s="26" t="s">
         <v>199</v>
       </c>
-      <c r="AR7" s="25" t="s">
+      <c r="AS7" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="AS7" s="26" t="s">
+      <c r="AT7" s="26" t="s">
         <v>201</v>
       </c>
-      <c r="AT7" s="26" t="s">
+      <c r="AU7" s="26" t="s">
         <v>202</v>
       </c>
-      <c r="AU7" s="26" t="s">
+      <c r="AV7" s="26" t="s">
         <v>203</v>
       </c>
-      <c r="AV7" s="26" t="s">
+      <c r="AW7" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="AW7" s="26" t="s">
+      <c r="AX7" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="AX7" s="9" t="s">
+      <c r="AY7" s="26" t="s">
         <v>206</v>
       </c>
-      <c r="AY7" s="9" t="s">
+      <c r="AZ7" s="26" t="s">
         <v>207</v>
       </c>
-      <c r="AZ7" s="26" t="s">
+      <c r="BA7" s="31" t="s">
+        <v>243</v>
+      </c>
+      <c r="BB7" s="26" t="s">
         <v>208</v>
       </c>
-      <c r="BA7" s="26" t="s">
+      <c r="BC7" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="BB7" s="31" t="s">
-        <v>245</v>
-      </c>
-      <c r="BC7" s="26" t="s">
+      <c r="BD7" s="26" t="s">
         <v>210</v>
       </c>
-      <c r="BD7" s="9" t="s">
+      <c r="BE7" s="26" t="s">
         <v>211</v>
       </c>
-      <c r="BE7" s="26" t="s">
+      <c r="BF7" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="BF7" s="26" t="s">
+      <c r="BG7" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="BG7" s="26" t="s">
+      <c r="BH7" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="BH7" s="26" t="s">
+      <c r="BI7" s="26" t="s">
         <v>215</v>
       </c>
-      <c r="BI7" s="26" t="s">
+      <c r="BJ7" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="BJ7" s="26" t="s">
+      <c r="BK7" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="BK7" s="9" t="s">
+      <c r="BL7" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="BL7" s="9" t="s">
+      <c r="BM7" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="BM7" s="9" t="s">
+      <c r="BN7" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="BN7" s="9" t="s">
+      <c r="BO7" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="BO7" s="9" t="s">
+      <c r="BP7" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="BP7" s="9" t="s">
+      <c r="BQ7" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="BQ7" s="9" t="s">
+      <c r="BR7" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="BR7" s="9" t="s">
+      <c r="BS7" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="BS7" s="9" t="s">
+      <c r="BT7" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="BT7" s="9" t="s">
+      <c r="BU7" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="BU7" s="9" t="s">
+      <c r="BV7" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="BV7" s="9" t="s">
+      <c r="BW7" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="BW7" s="9" t="s">
+      <c r="BX7" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="BX7" s="9" t="s">
+      <c r="BY7" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="BY7" s="27" t="s">
+      <c r="BZ7" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="BZ7" s="9" t="s">
+      <c r="CA7" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="CA7" s="9" t="s">
+      <c r="CB7" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="CB7" s="9" t="s">
+      <c r="CC7" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="CC7" s="9" t="s">
+      <c r="CD7" s="26" t="s">
         <v>236</v>
       </c>
-      <c r="CD7" s="9" t="s">
+      <c r="CE7" s="26" t="s">
         <v>237</v>
       </c>
-      <c r="CE7" s="26" t="s">
+      <c r="CF7" s="26" t="s">
         <v>238</v>
       </c>
-      <c r="CF7" s="26" t="s">
+      <c r="CG7" s="26" t="s">
         <v>239</v>
       </c>
-      <c r="CG7" s="26" t="s">
+      <c r="CH7" s="10" t="s">
         <v>240</v>
-      </c>
-      <c r="CH7" s="26" t="s">
-        <v>241</v>
-      </c>
-      <c r="CI7" s="10" t="s">
-        <v>242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>